<commit_message>
updated page data files
</commit_message>
<xml_diff>
--- a/page-data.xlsx
+++ b/page-data.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="pages" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">pages!$A$1:$E$993</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">pages!$A$1:$E$994</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1421" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1426" uniqueCount="299">
   <si>
     <t>-PAGE-</t>
   </si>
@@ -723,12 +723,12 @@
     <t>https://heatlabs.net/playground</t>
   </si>
   <si>
-    <t>https://heatlabs.net/playground/alpha-3-playtest</t>
-  </si>
-  <si>
     <t>https://heatlabs.net/playground/configurator</t>
   </si>
   <si>
+    <t>https://heatlabs.net/playground/countdown</t>
+  </si>
+  <si>
     <t>https://heatlabs.net/playground/game-data</t>
   </si>
   <si>
@@ -880,6 +880,9 @@
   </si>
   <si>
     <t>https://heatlabs.net/tournaments</t>
+  </si>
+  <si>
+    <t>https://heatlabs.net/tournaments/brackets</t>
   </si>
   <si>
     <t>https://heatlabs.net/tournaments/open-alpha-1-tournament</t>
@@ -1418,7 +1421,7 @@
       <c r="G3" s="10">
         <f>COUNTIF(B:B,"PENDING")
 </f>
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H3" s="10">
         <f>COUNTIF(B:B,"NOT INDEXED")
@@ -1428,7 +1431,7 @@
       <c r="I3" s="10">
         <f>COUNTIF(B:B,"INDEXED")
 </f>
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4">
@@ -1532,7 +1535,7 @@
       <c r="I7" s="10">
         <f>COUNTIF(C:C,"INDEXED")
 </f>
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8">
@@ -1626,7 +1629,7 @@
       <c r="G11" s="10">
         <f>COUNTIF(D:D,"UNKNOWN")
 </f>
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H11" s="10">
         <f>COUNTIF(D:D,"NOT HTTPS")
@@ -1730,7 +1733,7 @@
       <c r="G15" s="10">
         <f>COUNTIF(E:E,"UNKNOWN")
 </f>
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H15" s="10">
         <f>COUNTIF(E:E,"INVALID")
@@ -5657,7 +5660,7 @@
         <v>8</v>
       </c>
       <c r="C202" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D202" s="6" t="s">
         <v>15</v>
@@ -5678,7 +5681,7 @@
         <v>8</v>
       </c>
       <c r="C203" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D203" s="6" t="s">
         <v>15</v>
@@ -6053,10 +6056,10 @@
         <v>237</v>
       </c>
       <c r="B221" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C221" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D221" s="6" t="s">
         <v>15</v>
@@ -7145,10 +7148,10 @@
         <v>289</v>
       </c>
       <c r="B273" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C273" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D273" s="6" t="s">
         <v>15</v>
@@ -7211,7 +7214,7 @@
         <v>7</v>
       </c>
       <c r="C276" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D276" s="6" t="s">
         <v>15</v>
@@ -7229,7 +7232,7 @@
         <v>293</v>
       </c>
       <c r="B277" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C277" s="6" t="s">
         <v>8</v>
@@ -7250,7 +7253,7 @@
         <v>294</v>
       </c>
       <c r="B278" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C278" s="6" t="s">
         <v>8</v>
@@ -7313,16 +7316,16 @@
         <v>297</v>
       </c>
       <c r="B281" s="6" t="s">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="C281" s="6" t="s">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="D281" s="6" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="E281" s="6" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F281" s="2"/>
       <c r="G281" s="2"/>
@@ -7330,11 +7333,21 @@
       <c r="I281" s="2"/>
     </row>
     <row r="282">
-      <c r="A282" s="16"/>
-      <c r="B282" s="17"/>
-      <c r="C282" s="17"/>
-      <c r="D282" s="17"/>
-      <c r="E282" s="17"/>
+      <c r="A282" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="B282" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C282" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D282" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E282" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="F282" s="2"/>
       <c r="G282" s="2"/>
       <c r="H282" s="2"/>
@@ -15161,11 +15174,22 @@
       <c r="H993" s="2"/>
       <c r="I993" s="2"/>
     </row>
+    <row r="994">
+      <c r="A994" s="16"/>
+      <c r="B994" s="17"/>
+      <c r="C994" s="17"/>
+      <c r="D994" s="17"/>
+      <c r="E994" s="17"/>
+      <c r="F994" s="2"/>
+      <c r="G994" s="2"/>
+      <c r="H994" s="2"/>
+      <c r="I994" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$A$1:$E$993">
-    <sortState ref="A1:E993">
-      <sortCondition ref="A1:A993"/>
-      <sortCondition ref="D1:D993"/>
+  <autoFilter ref="$A$1:$E$994">
+    <sortState ref="A1:E994">
+      <sortCondition ref="A1:A994"/>
+      <sortCondition ref="D1:D994"/>
     </sortState>
   </autoFilter>
   <mergeCells count="4">
@@ -15175,13 +15199,13 @@
     <mergeCell ref="G13:I13"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:C993">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:C994">
       <formula1>"NOT INDEXED,NOT NEEDED,PENDING,INDEXED"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D993">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D994">
       <formula1>"NOT NEEDED,NOT HTTPS,UNKNOWN,HTTPS"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E993">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E994">
       <formula1>"NOT NEEDED,INVALID,UNKNOWN,VALID"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15466,7 +15490,8 @@
     <hyperlink r:id="rId278" ref="A279"/>
     <hyperlink r:id="rId279" ref="A280"/>
     <hyperlink r:id="rId280" ref="A281"/>
+    <hyperlink r:id="rId281" ref="A282"/>
   </hyperlinks>
-  <drawing r:id="rId281"/>
+  <drawing r:id="rId282"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated page data files with 1 new steam news post
</commit_message>
<xml_diff>
--- a/page-data.xlsx
+++ b/page-data.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="pages" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">pages!$A$1:$E$995</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">pages!$A$1:$E$996</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1431" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="301">
   <si>
     <t>-PAGE-</t>
   </si>
@@ -784,6 +784,9 @@
   </si>
   <si>
     <t>https://heatlabs.net/steam-news/heat-wrapped-2025-in-review</t>
+  </si>
+  <si>
+    <t>https://heatlabs.net/steam-news/human-machine-synergy</t>
   </si>
   <si>
     <t>https://heatlabs.net/steam-news/join-the-lodestar-program</t>
@@ -1424,7 +1427,7 @@
       <c r="G3" s="10">
         <f>COUNTIF(B:B,"PENDING")
 </f>
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H3" s="10">
         <f>COUNTIF(B:B,"NOT INDEXED")
@@ -1528,7 +1531,7 @@
       <c r="G7" s="10">
         <f>COUNTIF(C:C,"PENDING")
 </f>
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H7" s="10">
         <f>COUNTIF(C:C,"NOT INDEXED")
@@ -1632,7 +1635,7 @@
       <c r="G11" s="10">
         <f>COUNTIF(D:D,"UNKNOWN")
 </f>
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H11" s="10">
         <f>COUNTIF(D:D,"NOT HTTPS")
@@ -1736,7 +1739,7 @@
       <c r="G15" s="10">
         <f>COUNTIF(E:E,"UNKNOWN")
 </f>
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H15" s="10">
         <f>COUNTIF(E:E,"INVALID")
@@ -6475,20 +6478,20 @@
       <c r="I240" s="2"/>
     </row>
     <row r="241">
-      <c r="A241" s="5" t="s">
+      <c r="A241" s="14" t="s">
         <v>257</v>
       </c>
       <c r="B241" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C241" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D241" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E241" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F241" s="2"/>
       <c r="G241" s="2"/>
@@ -6496,20 +6499,20 @@
       <c r="I241" s="2"/>
     </row>
     <row r="242">
-      <c r="A242" s="14" t="s">
+      <c r="A242" s="5" t="s">
         <v>258</v>
       </c>
       <c r="B242" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C242" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D242" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E242" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F242" s="2"/>
       <c r="G242" s="2"/>
@@ -6517,20 +6520,20 @@
       <c r="I242" s="2"/>
     </row>
     <row r="243">
-      <c r="A243" s="5" t="s">
+      <c r="A243" s="14" t="s">
         <v>259</v>
       </c>
       <c r="B243" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C243" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D243" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E243" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F243" s="2"/>
       <c r="G243" s="2"/>
@@ -6548,10 +6551,10 @@
         <v>7</v>
       </c>
       <c r="D244" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E244" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F244" s="2"/>
       <c r="G244" s="2"/>
@@ -6569,10 +6572,10 @@
         <v>7</v>
       </c>
       <c r="D245" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E245" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F245" s="2"/>
       <c r="G245" s="2"/>
@@ -6590,10 +6593,10 @@
         <v>7</v>
       </c>
       <c r="D246" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E246" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F246" s="2"/>
       <c r="G246" s="2"/>
@@ -6727,7 +6730,7 @@
       <c r="I252" s="2"/>
     </row>
     <row r="253">
-      <c r="A253" s="15" t="s">
+      <c r="A253" s="5" t="s">
         <v>269</v>
       </c>
       <c r="B253" s="6" t="s">
@@ -6748,7 +6751,7 @@
       <c r="I253" s="2"/>
     </row>
     <row r="254">
-      <c r="A254" s="5" t="s">
+      <c r="A254" s="15" t="s">
         <v>270</v>
       </c>
       <c r="B254" s="6" t="s">
@@ -6989,10 +6992,10 @@
         <v>7</v>
       </c>
       <c r="D265" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E265" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F265" s="2"/>
       <c r="G265" s="2"/>
@@ -7010,10 +7013,10 @@
         <v>7</v>
       </c>
       <c r="D266" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E266" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F266" s="2"/>
       <c r="G266" s="2"/>
@@ -7157,10 +7160,10 @@
         <v>7</v>
       </c>
       <c r="D273" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E273" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F273" s="2"/>
       <c r="G273" s="2"/>
@@ -7172,16 +7175,16 @@
         <v>290</v>
       </c>
       <c r="B274" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C274" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D274" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E274" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F274" s="2"/>
       <c r="G274" s="2"/>
@@ -7193,10 +7196,10 @@
         <v>291</v>
       </c>
       <c r="B275" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C275" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D275" s="6" t="s">
         <v>15</v>
@@ -7259,7 +7262,7 @@
         <v>7</v>
       </c>
       <c r="C278" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D278" s="6" t="s">
         <v>15</v>
@@ -7277,7 +7280,7 @@
         <v>295</v>
       </c>
       <c r="B279" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C279" s="6" t="s">
         <v>8</v>
@@ -7298,7 +7301,7 @@
         <v>296</v>
       </c>
       <c r="B280" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C280" s="6" t="s">
         <v>8</v>
@@ -7361,16 +7364,16 @@
         <v>299</v>
       </c>
       <c r="B283" s="6" t="s">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="C283" s="6" t="s">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="D283" s="6" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="E283" s="6" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F283" s="2"/>
       <c r="G283" s="2"/>
@@ -7378,11 +7381,21 @@
       <c r="I283" s="2"/>
     </row>
     <row r="284">
-      <c r="A284" s="16"/>
-      <c r="B284" s="17"/>
-      <c r="C284" s="17"/>
-      <c r="D284" s="17"/>
-      <c r="E284" s="17"/>
+      <c r="A284" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="B284" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C284" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D284" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E284" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="F284" s="2"/>
       <c r="G284" s="2"/>
       <c r="H284" s="2"/>
@@ -15209,11 +15222,22 @@
       <c r="H995" s="2"/>
       <c r="I995" s="2"/>
     </row>
+    <row r="996">
+      <c r="A996" s="16"/>
+      <c r="B996" s="17"/>
+      <c r="C996" s="17"/>
+      <c r="D996" s="17"/>
+      <c r="E996" s="17"/>
+      <c r="F996" s="2"/>
+      <c r="G996" s="2"/>
+      <c r="H996" s="2"/>
+      <c r="I996" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$A$1:$E$995">
-    <sortState ref="A1:E995">
-      <sortCondition ref="A1:A995"/>
-      <sortCondition ref="D1:D995"/>
+  <autoFilter ref="$A$1:$E$996">
+    <sortState ref="A1:E996">
+      <sortCondition ref="A1:A996"/>
+      <sortCondition ref="D1:D996"/>
     </sortState>
   </autoFilter>
   <mergeCells count="4">
@@ -15223,13 +15247,13 @@
     <mergeCell ref="G13:I13"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:C995">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:C996">
       <formula1>"NOT INDEXED,NOT NEEDED,PENDING,INDEXED"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D995">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D996">
       <formula1>"NOT NEEDED,NOT HTTPS,UNKNOWN,HTTPS"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E995">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E996">
       <formula1>"NOT NEEDED,INVALID,UNKNOWN,VALID"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15516,7 +15540,8 @@
     <hyperlink r:id="rId280" ref="A281"/>
     <hyperlink r:id="rId281" ref="A282"/>
     <hyperlink r:id="rId282" ref="A283"/>
+    <hyperlink r:id="rId283" ref="A284"/>
   </hyperlinks>
-  <drawing r:id="rId283"/>
+  <drawing r:id="rId284"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated page data files with new guide structure
</commit_message>
<xml_diff>
--- a/page-data.xlsx
+++ b/page-data.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="pages" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">pages!$A$1:$E$866</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">pages!$A$1:$E$862</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="178">
   <si>
     <t>-PAGE-</t>
   </si>
@@ -282,25 +282,16 @@
     <t>https://heatlabs.net/guides</t>
   </si>
   <si>
-    <t>https://heatlabs.net/guides/general-guides</t>
-  </si>
-  <si>
-    <t>https://heatlabs.net/guides/general-guides/shell-crit-cone-mechanic</t>
-  </si>
-  <si>
-    <t>https://heatlabs.net/guides/map-guides</t>
-  </si>
-  <si>
-    <t>https://heatlabs.net/guides/tank-guides</t>
-  </si>
-  <si>
-    <t>https://heatlabs.net/guides/tank-guides/alvt-players-guide</t>
-  </si>
-  <si>
-    <t>https://heatlabs.net/guides/tank-guides/bat-4m-basic-guide</t>
-  </si>
-  <si>
-    <t>https://heatlabs.net/guides/tank-guides/xm1-v-build-guide</t>
+    <t>https://heatlabs.net/guides/shell-crit-cone-mechanic</t>
+  </si>
+  <si>
+    <t>https://heatlabs.net/guides/alvt-players-guide</t>
+  </si>
+  <si>
+    <t>https://heatlabs.net/guides/bat-4m-basic-guide</t>
+  </si>
+  <si>
+    <t>https://heatlabs.net/guides/xm1-v-build-guide</t>
   </si>
   <si>
     <t>https://heatlabs.net/legal</t>
@@ -1067,7 +1058,7 @@
       <c r="G3" s="10">
         <f>COUNTIF(B:B,"PENDING")
 </f>
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H3" s="10">
         <f>COUNTIF(B:B,"NOT INDEXED")
@@ -1077,7 +1068,7 @@
       <c r="I3" s="10">
         <f>COUNTIF(B:B,"INDEXED")
 </f>
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4">
@@ -1171,7 +1162,7 @@
       <c r="G7" s="10">
         <f>COUNTIF(C:C,"PENDING")
 </f>
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H7" s="10">
         <f>COUNTIF(C:C,"NOT INDEXED")
@@ -1181,7 +1172,7 @@
       <c r="I7" s="10">
         <f>COUNTIF(C:C,"INDEXED")
 </f>
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8">
@@ -2585,10 +2576,10 @@
         <v>89</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D74" s="6" t="s">
         <v>15</v>
@@ -2602,7 +2593,7 @@
       <c r="I74" s="2"/>
     </row>
     <row r="75">
-      <c r="A75" s="14" t="s">
+      <c r="A75" s="5" t="s">
         <v>90</v>
       </c>
       <c r="B75" s="6" t="s">
@@ -2623,14 +2614,14 @@
       <c r="I75" s="2"/>
     </row>
     <row r="76">
-      <c r="A76" s="14" t="s">
-        <v>90</v>
+      <c r="A76" s="5" t="s">
+        <v>91</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D76" s="6" t="s">
         <v>15</v>
@@ -2645,7 +2636,7 @@
     </row>
     <row r="77">
       <c r="A77" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B77" s="6" t="s">
         <v>7</v>
@@ -2666,7 +2657,7 @@
     </row>
     <row r="78">
       <c r="A78" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B78" s="6" t="s">
         <v>7</v>
@@ -2675,10 +2666,10 @@
         <v>7</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
@@ -2686,14 +2677,14 @@
       <c r="I78" s="2"/>
     </row>
     <row r="79">
-      <c r="A79" s="14" t="s">
-        <v>93</v>
+      <c r="A79" s="5" t="s">
+        <v>94</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>15</v>
@@ -2707,11 +2698,11 @@
       <c r="I79" s="2"/>
     </row>
     <row r="80">
-      <c r="A80" s="5" t="s">
-        <v>94</v>
+      <c r="A80" s="14" t="s">
+        <v>95</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C80" s="6" t="s">
         <v>7</v>
@@ -2729,7 +2720,7 @@
     </row>
     <row r="81">
       <c r="A81" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B81" s="6" t="s">
         <v>7</v>
@@ -2738,10 +2729,10 @@
         <v>7</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
@@ -2750,19 +2741,19 @@
     </row>
     <row r="82">
       <c r="A82" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
@@ -2771,7 +2762,7 @@
     </row>
     <row r="83">
       <c r="A83" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B83" s="6" t="s">
         <v>7</v>
@@ -2780,10 +2771,10 @@
         <v>7</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
@@ -2791,14 +2782,14 @@
       <c r="I83" s="2"/>
     </row>
     <row r="84">
-      <c r="A84" s="14" t="s">
-        <v>98</v>
+      <c r="A84" s="5" t="s">
+        <v>99</v>
       </c>
       <c r="B84" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C84" s="6" t="s">
         <v>8</v>
-      </c>
-      <c r="C84" s="6" t="s">
-        <v>7</v>
       </c>
       <c r="D84" s="6" t="s">
         <v>15</v>
@@ -2813,10 +2804,10 @@
     </row>
     <row r="85">
       <c r="A85" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C85" s="6" t="s">
         <v>7</v>
@@ -2834,19 +2825,19 @@
     </row>
     <row r="86">
       <c r="A86" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F86" s="2"/>
       <c r="G86" s="2"/>
@@ -2855,19 +2846,19 @@
     </row>
     <row r="87">
       <c r="A87" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C87" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F87" s="2"/>
       <c r="G87" s="2"/>
@@ -2876,13 +2867,13 @@
     </row>
     <row r="88">
       <c r="A88" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D88" s="6" t="s">
         <v>15</v>
@@ -2897,19 +2888,19 @@
     </row>
     <row r="89">
       <c r="A89" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B89" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C89" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C89" s="6" t="s">
-        <v>7</v>
-      </c>
       <c r="D89" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
@@ -2918,7 +2909,7 @@
     </row>
     <row r="90">
       <c r="A90" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B90" s="6" t="s">
         <v>7</v>
@@ -2927,10 +2918,10 @@
         <v>7</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
@@ -2939,10 +2930,10 @@
     </row>
     <row r="91">
       <c r="A91" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C91" s="6" t="s">
         <v>7</v>
@@ -2960,13 +2951,13 @@
     </row>
     <row r="92">
       <c r="A92" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B92" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D92" s="6" t="s">
         <v>15</v>
@@ -2981,13 +2972,13 @@
     </row>
     <row r="93">
       <c r="A93" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B93" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D93" s="6" t="s">
         <v>15</v>
@@ -3002,7 +2993,7 @@
     </row>
     <row r="94">
       <c r="A94" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B94" s="6" t="s">
         <v>7</v>
@@ -3023,10 +3014,10 @@
     </row>
     <row r="95">
       <c r="A95" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C95" s="6" t="s">
         <v>7</v>
@@ -3044,13 +3035,13 @@
     </row>
     <row r="96">
       <c r="A96" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B96" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D96" s="6" t="s">
         <v>15</v>
@@ -3065,10 +3056,10 @@
     </row>
     <row r="97">
       <c r="A97" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C97" s="6" t="s">
         <v>7</v>
@@ -3086,10 +3077,10 @@
     </row>
     <row r="98">
       <c r="A98" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C98" s="6" t="s">
         <v>7</v>
@@ -3107,13 +3098,13 @@
     </row>
     <row r="99">
       <c r="A99" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B99" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D99" s="6" t="s">
         <v>15</v>
@@ -3128,10 +3119,10 @@
     </row>
     <row r="100">
       <c r="A100" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C100" s="6" t="s">
         <v>7</v>
@@ -3149,10 +3140,10 @@
     </row>
     <row r="101">
       <c r="A101" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C101" s="6" t="s">
         <v>7</v>
@@ -3170,19 +3161,19 @@
     </row>
     <row r="102">
       <c r="A102" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C102" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F102" s="2"/>
       <c r="G102" s="2"/>
@@ -3191,19 +3182,19 @@
     </row>
     <row r="103">
       <c r="A103" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B103" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C103" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F103" s="2"/>
       <c r="G103" s="2"/>
@@ -3212,7 +3203,7 @@
     </row>
     <row r="104">
       <c r="A104" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B104" s="6" t="s">
         <v>7</v>
@@ -3221,10 +3212,10 @@
         <v>7</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F104" s="2"/>
       <c r="G104" s="2"/>
@@ -3233,7 +3224,7 @@
     </row>
     <row r="105">
       <c r="A105" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B105" s="6" t="s">
         <v>7</v>
@@ -3254,19 +3245,19 @@
     </row>
     <row r="106">
       <c r="A106" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C106" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F106" s="2"/>
       <c r="G106" s="2"/>
@@ -3274,8 +3265,8 @@
       <c r="I106" s="2"/>
     </row>
     <row r="107">
-      <c r="A107" s="5" t="s">
-        <v>121</v>
+      <c r="A107" s="14" t="s">
+        <v>122</v>
       </c>
       <c r="B107" s="6" t="s">
         <v>8</v>
@@ -3284,10 +3275,10 @@
         <v>7</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E107" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F107" s="2"/>
       <c r="G107" s="2"/>
@@ -3296,7 +3287,7 @@
     </row>
     <row r="108">
       <c r="A108" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B108" s="6" t="s">
         <v>7</v>
@@ -3305,10 +3296,10 @@
         <v>7</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F108" s="2"/>
       <c r="G108" s="2"/>
@@ -3317,7 +3308,7 @@
     </row>
     <row r="109">
       <c r="A109" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B109" s="6" t="s">
         <v>7</v>
@@ -3337,14 +3328,14 @@
       <c r="I109" s="2"/>
     </row>
     <row r="110">
-      <c r="A110" s="5" t="s">
-        <v>124</v>
+      <c r="A110" s="14" t="s">
+        <v>125</v>
       </c>
       <c r="B110" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C110" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D110" s="6" t="s">
         <v>15</v>
@@ -3358,11 +3349,11 @@
       <c r="I110" s="2"/>
     </row>
     <row r="111">
-      <c r="A111" s="14" t="s">
-        <v>125</v>
+      <c r="A111" s="5" t="s">
+        <v>126</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C111" s="6" t="s">
         <v>7</v>
@@ -3380,7 +3371,7 @@
     </row>
     <row r="112">
       <c r="A112" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B112" s="6" t="s">
         <v>7</v>
@@ -3401,7 +3392,7 @@
     </row>
     <row r="113">
       <c r="A113" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B113" s="6" t="s">
         <v>7</v>
@@ -3422,7 +3413,7 @@
     </row>
     <row r="114">
       <c r="A114" s="14" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B114" s="6" t="s">
         <v>8</v>
@@ -3443,7 +3434,7 @@
     </row>
     <row r="115">
       <c r="A115" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B115" s="6" t="s">
         <v>7</v>
@@ -3463,14 +3454,14 @@
       <c r="I115" s="2"/>
     </row>
     <row r="116">
-      <c r="A116" s="5" t="s">
-        <v>130</v>
+      <c r="A116" s="14" t="s">
+        <v>131</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C116" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D116" s="6" t="s">
         <v>15</v>
@@ -3485,10 +3476,10 @@
     </row>
     <row r="117">
       <c r="A117" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B117" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C117" s="6" t="s">
         <v>7</v>
@@ -3505,20 +3496,20 @@
       <c r="I117" s="2"/>
     </row>
     <row r="118">
-      <c r="A118" s="14" t="s">
-        <v>132</v>
+      <c r="A118" s="5" t="s">
+        <v>133</v>
       </c>
       <c r="B118" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C118" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F118" s="2"/>
       <c r="G118" s="2"/>
@@ -3527,10 +3518,10 @@
     </row>
     <row r="119">
       <c r="A119" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B119" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C119" s="6" t="s">
         <v>7</v>
@@ -3547,14 +3538,14 @@
       <c r="I119" s="2"/>
     </row>
     <row r="120">
-      <c r="A120" s="14" t="s">
-        <v>134</v>
+      <c r="A120" s="5" t="s">
+        <v>135</v>
       </c>
       <c r="B120" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C120" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D120" s="6" t="s">
         <v>15</v>
@@ -3569,10 +3560,10 @@
     </row>
     <row r="121">
       <c r="A121" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B121" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C121" s="6" t="s">
         <v>7</v>
@@ -3590,10 +3581,10 @@
     </row>
     <row r="122">
       <c r="A122" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B122" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C122" s="6" t="s">
         <v>7</v>
@@ -3611,19 +3602,19 @@
     </row>
     <row r="123">
       <c r="A123" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B123" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C123" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D123" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F123" s="2"/>
       <c r="G123" s="2"/>
@@ -3632,7 +3623,7 @@
     </row>
     <row r="124">
       <c r="A124" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B124" s="6" t="s">
         <v>7</v>
@@ -3641,10 +3632,10 @@
         <v>7</v>
       </c>
       <c r="D124" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F124" s="2"/>
       <c r="G124" s="2"/>
@@ -3652,8 +3643,8 @@
       <c r="I124" s="2"/>
     </row>
     <row r="125">
-      <c r="A125" s="5" t="s">
-        <v>139</v>
+      <c r="A125" s="15" t="s">
+        <v>140</v>
       </c>
       <c r="B125" s="6" t="s">
         <v>7</v>
@@ -3674,10 +3665,10 @@
     </row>
     <row r="126">
       <c r="A126" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B126" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C126" s="6" t="s">
         <v>7</v>
@@ -3695,7 +3686,7 @@
     </row>
     <row r="127">
       <c r="A127" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B127" s="6" t="s">
         <v>7</v>
@@ -3704,10 +3695,10 @@
         <v>7</v>
       </c>
       <c r="D127" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F127" s="2"/>
       <c r="G127" s="2"/>
@@ -3716,7 +3707,7 @@
     </row>
     <row r="128">
       <c r="A128" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B128" s="6" t="s">
         <v>7</v>
@@ -3725,10 +3716,10 @@
         <v>7</v>
       </c>
       <c r="D128" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F128" s="2"/>
       <c r="G128" s="2"/>
@@ -3736,8 +3727,8 @@
       <c r="I128" s="2"/>
     </row>
     <row r="129">
-      <c r="A129" s="15" t="s">
-        <v>143</v>
+      <c r="A129" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="B129" s="6" t="s">
         <v>7</v>
@@ -3758,7 +3749,7 @@
     </row>
     <row r="130">
       <c r="A130" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B130" s="6" t="s">
         <v>7</v>
@@ -3767,10 +3758,10 @@
         <v>7</v>
       </c>
       <c r="D130" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F130" s="2"/>
       <c r="G130" s="2"/>
@@ -3779,7 +3770,7 @@
     </row>
     <row r="131">
       <c r="A131" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B131" s="6" t="s">
         <v>7</v>
@@ -3800,7 +3791,7 @@
     </row>
     <row r="132">
       <c r="A132" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B132" s="6" t="s">
         <v>7</v>
@@ -3821,7 +3812,7 @@
     </row>
     <row r="133">
       <c r="A133" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B133" s="6" t="s">
         <v>7</v>
@@ -3842,13 +3833,13 @@
     </row>
     <row r="134">
       <c r="A134" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B134" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C134" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D134" s="6" t="s">
         <v>15</v>
@@ -3863,7 +3854,7 @@
     </row>
     <row r="135">
       <c r="A135" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B135" s="6" t="s">
         <v>7</v>
@@ -3883,14 +3874,14 @@
       <c r="I135" s="2"/>
     </row>
     <row r="136">
-      <c r="A136" s="5" t="s">
-        <v>150</v>
+      <c r="A136" s="14" t="s">
+        <v>151</v>
       </c>
       <c r="B136" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C136" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D136" s="6" t="s">
         <v>15</v>
@@ -3905,7 +3896,7 @@
     </row>
     <row r="137">
       <c r="A137" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B137" s="6" t="s">
         <v>7</v>
@@ -3926,13 +3917,13 @@
     </row>
     <row r="138">
       <c r="A138" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B138" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C138" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D138" s="6" t="s">
         <v>15</v>
@@ -3947,7 +3938,7 @@
     </row>
     <row r="139">
       <c r="A139" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B139" s="6" t="s">
         <v>7</v>
@@ -3967,14 +3958,14 @@
       <c r="I139" s="2"/>
     </row>
     <row r="140">
-      <c r="A140" s="14" t="s">
-        <v>154</v>
+      <c r="A140" s="5" t="s">
+        <v>155</v>
       </c>
       <c r="B140" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C140" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D140" s="6" t="s">
         <v>15</v>
@@ -3989,7 +3980,7 @@
     </row>
     <row r="141">
       <c r="A141" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B141" s="6" t="s">
         <v>7</v>
@@ -4010,7 +4001,7 @@
     </row>
     <row r="142">
       <c r="A142" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B142" s="6" t="s">
         <v>7</v>
@@ -4031,7 +4022,7 @@
     </row>
     <row r="143">
       <c r="A143" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B143" s="6" t="s">
         <v>7</v>
@@ -4052,7 +4043,7 @@
     </row>
     <row r="144">
       <c r="A144" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B144" s="6" t="s">
         <v>7</v>
@@ -4073,7 +4064,7 @@
     </row>
     <row r="145">
       <c r="A145" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B145" s="6" t="s">
         <v>7</v>
@@ -4094,7 +4085,7 @@
     </row>
     <row r="146">
       <c r="A146" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B146" s="6" t="s">
         <v>7</v>
@@ -4103,10 +4094,10 @@
         <v>7</v>
       </c>
       <c r="D146" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E146" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F146" s="2"/>
       <c r="G146" s="2"/>
@@ -4115,7 +4106,7 @@
     </row>
     <row r="147">
       <c r="A147" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B147" s="6" t="s">
         <v>7</v>
@@ -4136,7 +4127,7 @@
     </row>
     <row r="148">
       <c r="A148" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B148" s="6" t="s">
         <v>7</v>
@@ -4156,14 +4147,14 @@
       <c r="I148" s="2"/>
     </row>
     <row r="149">
-      <c r="A149" s="5" t="s">
-        <v>163</v>
+      <c r="A149" s="14" t="s">
+        <v>164</v>
       </c>
       <c r="B149" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C149" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D149" s="6" t="s">
         <v>15</v>
@@ -4178,7 +4169,7 @@
     </row>
     <row r="150">
       <c r="A150" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B150" s="6" t="s">
         <v>7</v>
@@ -4187,10 +4178,10 @@
         <v>7</v>
       </c>
       <c r="D150" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E150" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F150" s="2"/>
       <c r="G150" s="2"/>
@@ -4199,7 +4190,7 @@
     </row>
     <row r="151">
       <c r="A151" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B151" s="6" t="s">
         <v>7</v>
@@ -4220,7 +4211,7 @@
     </row>
     <row r="152">
       <c r="A152" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B152" s="6" t="s">
         <v>7</v>
@@ -4229,10 +4220,10 @@
         <v>7</v>
       </c>
       <c r="D152" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E152" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F152" s="2"/>
       <c r="G152" s="2"/>
@@ -4240,14 +4231,14 @@
       <c r="I152" s="2"/>
     </row>
     <row r="153">
-      <c r="A153" s="14" t="s">
-        <v>167</v>
+      <c r="A153" s="5" t="s">
+        <v>168</v>
       </c>
       <c r="B153" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C153" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D153" s="6" t="s">
         <v>15</v>
@@ -4262,7 +4253,7 @@
     </row>
     <row r="154">
       <c r="A154" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B154" s="6" t="s">
         <v>7</v>
@@ -4283,7 +4274,7 @@
     </row>
     <row r="155">
       <c r="A155" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B155" s="6" t="s">
         <v>7</v>
@@ -4304,7 +4295,7 @@
     </row>
     <row r="156">
       <c r="A156" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B156" s="6" t="s">
         <v>7</v>
@@ -4313,10 +4304,10 @@
         <v>7</v>
       </c>
       <c r="D156" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E156" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F156" s="2"/>
       <c r="G156" s="2"/>
@@ -4325,13 +4316,13 @@
     </row>
     <row r="157">
       <c r="A157" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B157" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C157" s="6" t="s">
         <v>8</v>
-      </c>
-      <c r="C157" s="6" t="s">
-        <v>7</v>
       </c>
       <c r="D157" s="6" t="s">
         <v>15</v>
@@ -4346,13 +4337,13 @@
     </row>
     <row r="158">
       <c r="A158" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B158" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C158" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D158" s="6" t="s">
         <v>15</v>
@@ -4367,13 +4358,13 @@
     </row>
     <row r="159">
       <c r="A159" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B159" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C159" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D159" s="6" t="s">
         <v>15</v>
@@ -4388,13 +4379,13 @@
     </row>
     <row r="160">
       <c r="A160" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B160" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C160" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D160" s="6" t="s">
         <v>15</v>
@@ -4409,7 +4400,7 @@
     </row>
     <row r="161">
       <c r="A161" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B161" s="6" t="s">
         <v>7</v>
@@ -4430,19 +4421,19 @@
     </row>
     <row r="162">
       <c r="A162" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B162" s="6" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="C162" s="6" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="D162" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E162" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="F162" s="2"/>
       <c r="G162" s="2"/>
@@ -4450,84 +4441,44 @@
       <c r="I162" s="2"/>
     </row>
     <row r="163">
-      <c r="A163" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="B163" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C163" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D163" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E163" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A163" s="16"/>
+      <c r="B163" s="17"/>
+      <c r="C163" s="17"/>
+      <c r="D163" s="17"/>
+      <c r="E163" s="17"/>
       <c r="F163" s="2"/>
       <c r="G163" s="2"/>
       <c r="H163" s="2"/>
       <c r="I163" s="2"/>
     </row>
     <row r="164">
-      <c r="A164" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="B164" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C164" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D164" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E164" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A164" s="16"/>
+      <c r="B164" s="17"/>
+      <c r="C164" s="17"/>
+      <c r="D164" s="17"/>
+      <c r="E164" s="17"/>
       <c r="F164" s="2"/>
       <c r="G164" s="2"/>
       <c r="H164" s="2"/>
       <c r="I164" s="2"/>
     </row>
     <row r="165">
-      <c r="A165" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="B165" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C165" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D165" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E165" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A165" s="16"/>
+      <c r="B165" s="17"/>
+      <c r="C165" s="17"/>
+      <c r="D165" s="17"/>
+      <c r="E165" s="17"/>
       <c r="F165" s="2"/>
       <c r="G165" s="2"/>
       <c r="H165" s="2"/>
       <c r="I165" s="2"/>
     </row>
     <row r="166">
-      <c r="A166" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="B166" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C166" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D166" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E166" s="6" t="s">
-        <v>35</v>
-      </c>
+      <c r="A166" s="16"/>
+      <c r="B166" s="17"/>
+      <c r="C166" s="17"/>
+      <c r="D166" s="17"/>
+      <c r="E166" s="17"/>
       <c r="F166" s="2"/>
       <c r="G166" s="2"/>
       <c r="H166" s="2"/>
@@ -12189,55 +12140,11 @@
       <c r="H862" s="2"/>
       <c r="I862" s="2"/>
     </row>
-    <row r="863">
-      <c r="A863" s="16"/>
-      <c r="B863" s="17"/>
-      <c r="C863" s="17"/>
-      <c r="D863" s="17"/>
-      <c r="E863" s="17"/>
-      <c r="F863" s="2"/>
-      <c r="G863" s="2"/>
-      <c r="H863" s="2"/>
-      <c r="I863" s="2"/>
-    </row>
-    <row r="864">
-      <c r="A864" s="16"/>
-      <c r="B864" s="17"/>
-      <c r="C864" s="17"/>
-      <c r="D864" s="17"/>
-      <c r="E864" s="17"/>
-      <c r="F864" s="2"/>
-      <c r="G864" s="2"/>
-      <c r="H864" s="2"/>
-      <c r="I864" s="2"/>
-    </row>
-    <row r="865">
-      <c r="A865" s="16"/>
-      <c r="B865" s="17"/>
-      <c r="C865" s="17"/>
-      <c r="D865" s="17"/>
-      <c r="E865" s="17"/>
-      <c r="F865" s="2"/>
-      <c r="G865" s="2"/>
-      <c r="H865" s="2"/>
-      <c r="I865" s="2"/>
-    </row>
-    <row r="866">
-      <c r="A866" s="16"/>
-      <c r="B866" s="17"/>
-      <c r="C866" s="17"/>
-      <c r="D866" s="17"/>
-      <c r="E866" s="17"/>
-      <c r="F866" s="2"/>
-      <c r="G866" s="2"/>
-      <c r="H866" s="2"/>
-      <c r="I866" s="2"/>
-    </row>
   </sheetData>
-  <autoFilter ref="$A$1:$E$866">
-    <sortState ref="A1:E866">
-      <sortCondition ref="A1:A866"/>
-      <sortCondition ref="D1:D866"/>
+  <autoFilter ref="$A$1:$E$862">
+    <sortState ref="A1:E862">
+      <sortCondition ref="A1:A862"/>
+      <sortCondition ref="D1:D862"/>
     </sortState>
   </autoFilter>
   <mergeCells count="4">
@@ -12247,13 +12154,13 @@
     <mergeCell ref="G11:I11"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:C866">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:C862">
       <formula1>"NOT INDEXED,NOT NEEDED,PENDING,INDEXED"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D866">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D862">
       <formula1>"NOT NEEDED,NOT HTTPS,UNKNOWN,HTTPS"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E866">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E862">
       <formula1>"NOT NEEDED,INVALID,UNKNOWN,VALID"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12419,11 +12326,7 @@
     <hyperlink r:id="rId159" ref="A160"/>
     <hyperlink r:id="rId160" ref="A161"/>
     <hyperlink r:id="rId161" ref="A162"/>
-    <hyperlink r:id="rId162" ref="A163"/>
-    <hyperlink r:id="rId163" ref="A164"/>
-    <hyperlink r:id="rId164" ref="A165"/>
-    <hyperlink r:id="rId165" ref="A166"/>
   </hyperlinks>
-  <drawing r:id="rId166"/>
+  <drawing r:id="rId162"/>
 </worksheet>
 </file>
</xml_diff>